<commit_message>
added untracked files and html doc
</commit_message>
<xml_diff>
--- a/results/final_output.xlsx
+++ b/results/final_output.xlsx
@@ -428,31 +428,31 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.792422575066813</v>
+        <v>0.727990189913219</v>
       </c>
       <c r="D2">
-        <v>0.775325410299943</v>
+        <v>0.663532888944787</v>
       </c>
       <c r="E2">
-        <v>0.809520814991825</v>
+        <v>0.79244749088165</v>
       </c>
       <c r="F2">
-        <v>0.802786639755192</v>
+        <v>0.76173115795553</v>
       </c>
       <c r="G2">
-        <v>0.775325410299943</v>
+        <v>0.663532888944787</v>
       </c>
       <c r="H2">
-        <v>0.788817094235813</v>
+        <v>0.7092491765813</v>
       </c>
       <c r="I2">
-        <v>0.805930325950338</v>
+        <v>0.749208609076493</v>
       </c>
       <c r="J2">
-        <v>0.323995680207336</v>
+        <v>0.321324857062792</v>
       </c>
       <c r="K2">
-        <v>0.7806663205480489</v>
+        <v>0.6810934675961788</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -472,31 +472,31 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.730893146206918</v>
+        <v>0.74312979499434</v>
       </c>
       <c r="D3">
-        <v>0.692474469756481</v>
+        <v>0.730254056093573</v>
       </c>
       <c r="E3">
-        <v>0.769337190290529</v>
+        <v>0.7560055338951071</v>
       </c>
       <c r="F3">
-        <v>0.7502553278409479</v>
+        <v>0.749556236888817</v>
       </c>
       <c r="G3">
-        <v>0.692474469756481</v>
+        <v>0.730254056093573</v>
       </c>
       <c r="H3">
-        <v>0.7202078465334401</v>
+        <v>0.73977926069853</v>
       </c>
       <c r="I3">
-        <v>0.786542604876708</v>
+        <v>0.787473773359911</v>
       </c>
       <c r="J3">
-        <v>0.32277354161338</v>
+        <v>0.324240239035571</v>
       </c>
       <c r="K3">
-        <v>0.7033075047550967</v>
+        <v>0.7340345509826106</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -516,31 +516,31 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.713538954536351</v>
+        <v>0.713839375125175</v>
       </c>
       <c r="D4">
-        <v>0.440472249806907</v>
+        <v>0.441299790356394</v>
       </c>
       <c r="E4">
         <v>0.869167400327003</v>
       </c>
       <c r="F4">
-        <v>0.657389872375463</v>
+        <v>0.6578125</v>
       </c>
       <c r="G4">
-        <v>0.440472249806907</v>
+        <v>0.441299790356394</v>
       </c>
       <c r="H4">
-        <v>0.527501569158601</v>
+        <v>0.52823086574655</v>
       </c>
       <c r="I4">
-        <v>0.685879150832447</v>
+        <v>0.685889106090095</v>
       </c>
       <c r="J4">
-        <v>0.314424734355705</v>
+        <v>0.314441358403384</v>
       </c>
       <c r="K4">
-        <v>0.4715944665619202</v>
+        <v>0.4723967684021543</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -560,31 +560,31 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.836370919287002</v>
+        <v>0.838814340076107</v>
       </c>
       <c r="D5">
-        <v>0.664735738717864</v>
+        <v>0.671466401853691</v>
       </c>
       <c r="E5">
         <v>0.934190667840523</v>
       </c>
       <c r="F5">
-        <v>0.8520011313817</v>
+        <v>0.853266965787998</v>
       </c>
       <c r="G5">
-        <v>0.664735738717864</v>
+        <v>0.671466401853691</v>
       </c>
       <c r="H5">
-        <v>0.746807983141192</v>
+        <v>0.75152824945971</v>
       </c>
       <c r="I5">
-        <v>0.799463203279194</v>
+        <v>0.802828534847107</v>
       </c>
       <c r="J5">
-        <v>0.316754488813326</v>
+        <v>0.316904116963993</v>
       </c>
       <c r="K5">
-        <v>0.695300417791935</v>
+        <v>0.7013530333763601</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -604,31 +604,31 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.781175323858634</v>
+        <v>0.717897119859137</v>
       </c>
       <c r="D6">
-        <v>0.687806565211923</v>
+        <v>0.567004150421331</v>
       </c>
       <c r="E6">
-        <v>0.874544082505345</v>
+        <v>0.868790089296944</v>
       </c>
       <c r="F6">
-        <v>0.84573748308525</v>
+        <v>0.812077816806269</v>
       </c>
       <c r="G6">
-        <v>0.687806565211923</v>
+        <v>0.567004150421331</v>
       </c>
       <c r="H6">
-        <v>0.758639823822157</v>
+        <v>0.667765228661359</v>
       </c>
       <c r="I6">
-        <v>0.809603933097738</v>
+        <v>0.7311769816038211</v>
       </c>
       <c r="J6">
-        <v>0.319762499117466</v>
+        <v>0.316828430168703</v>
       </c>
       <c r="K6">
-        <v>0.7144910210934079</v>
+        <v>0.6034251984312888</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -648,31 +648,31 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.848006540057854</v>
+        <v>0.852361338196453</v>
       </c>
       <c r="D7">
-        <v>0.792793359325871</v>
+        <v>0.8015029556030689</v>
       </c>
       <c r="E7">
         <v>0.903219720789838</v>
       </c>
       <c r="F7">
-        <v>0.891205994627457</v>
+        <v>0.892260842171585</v>
       </c>
       <c r="G7">
-        <v>0.792793359325871</v>
+        <v>0.8015029556030689</v>
       </c>
       <c r="H7">
-        <v>0.839124068157614</v>
+        <v>0.844450333758468</v>
       </c>
       <c r="I7">
-        <v>0.857661756978004</v>
+        <v>0.86207230876102</v>
       </c>
       <c r="J7">
-        <v>0.3218357049313</v>
+        <v>0.322078182126949</v>
       </c>
       <c r="K7">
-        <v>0.8106978419116702</v>
+        <v>0.8181468048913569</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -780,31 +780,31 @@
         </is>
       </c>
       <c r="C10">
-        <v>0.817638736047791</v>
+        <v>0.781002389636524</v>
       </c>
       <c r="D10">
-        <v>0.7797065337763009</v>
+        <v>0.780104055663512</v>
       </c>
       <c r="E10">
-        <v>0.867479083303019</v>
+        <v>0.781906504321494</v>
       </c>
       <c r="F10">
-        <v>0.885461862541659</v>
+        <v>0.782605961514275</v>
       </c>
       <c r="G10">
-        <v>0.7797065337763009</v>
+        <v>0.780104055663512</v>
       </c>
       <c r="H10">
-        <v>0.829225922327238</v>
+        <v>0.7813530058075659</v>
       </c>
       <c r="I10">
-        <v>0.882065102377162</v>
+        <v>0.865626159324245</v>
       </c>
       <c r="J10">
-        <v>0.880248922170858</v>
+        <v>0.857845706572228</v>
       </c>
       <c r="K10">
-        <v>0.7987871980758536</v>
+        <v>0.7806031562837147</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -824,31 +824,31 @@
         </is>
       </c>
       <c r="C11">
-        <v>0.875214131920979</v>
+        <v>0.893346748836624</v>
       </c>
       <c r="D11">
-        <v>0.886651341988539</v>
+        <v>0.883436523018452</v>
       </c>
       <c r="E11">
-        <v>0.864424897684931</v>
+        <v>0.90378284164999</v>
       </c>
       <c r="F11">
-        <v>0.860518460329929</v>
+        <v>0.906269651616149</v>
       </c>
       <c r="G11">
-        <v>0.886651341988539</v>
+        <v>0.883436523018452</v>
       </c>
       <c r="H11">
-        <v>0.8733894629417021</v>
+        <v>0.894707434424957</v>
       </c>
       <c r="I11">
-        <v>0.946890434468859</v>
+        <v>0.952021416794455</v>
       </c>
       <c r="J11">
-        <v>0.949375750700591</v>
+        <v>0.955099990717249</v>
       </c>
       <c r="K11">
-        <v>0.8812985525155592</v>
+        <v>0.8879106390319642</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -868,31 +868,31 @@
         </is>
       </c>
       <c r="C12">
-        <v>0.78133386741438</v>
+        <v>0.792028840376527</v>
       </c>
       <c r="D12">
-        <v>0.6692177669264719</v>
+        <v>0.692529593156272</v>
       </c>
       <c r="E12">
-        <v>0.864731768650461</v>
+        <v>0.859106759656652</v>
       </c>
       <c r="F12">
-        <v>0.786329030122476</v>
+        <v>0.7681783074037291</v>
       </c>
       <c r="G12">
-        <v>0.6692177669264719</v>
+        <v>0.692529593156272</v>
       </c>
       <c r="H12">
-        <v>0.723062094155844</v>
+        <v>0.728395061728395</v>
       </c>
       <c r="I12">
-        <v>0.849356142714188</v>
+        <v>0.850387244777828</v>
       </c>
       <c r="J12">
-        <v>0.730279596897466</v>
+        <v>0.736133218633207</v>
       </c>
       <c r="K12">
-        <v>0.6897636423469289</v>
+        <v>0.7064434297311012</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -912,31 +912,31 @@
         </is>
       </c>
       <c r="C13">
-        <v>0.9192269176847589</v>
+        <v>0.919467254155818</v>
       </c>
       <c r="D13">
-        <v>0.867790594498669</v>
+        <v>0.86771990197612</v>
       </c>
       <c r="E13">
-        <v>0.95125280296383</v>
+        <v>0.951741406783519</v>
       </c>
       <c r="F13">
-        <v>0.917245945051308</v>
+        <v>0.91812865497076</v>
       </c>
       <c r="G13">
-        <v>0.867790594498669</v>
+        <v>0.86771990197612</v>
       </c>
       <c r="H13">
-        <v>0.891833176880783</v>
+        <v>0.892212840101863</v>
       </c>
       <c r="I13">
-        <v>0.9696788152172759</v>
+        <v>0.970441063743721</v>
       </c>
       <c r="J13">
-        <v>0.950413064293074</v>
+        <v>0.950374049621296</v>
       </c>
       <c r="K13">
-        <v>0.877250374622739</v>
+        <v>0.8773539149322033</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -956,31 +956,31 @@
         </is>
       </c>
       <c r="C14">
-        <v>0.844846560181109</v>
+        <v>0.831923657401585</v>
       </c>
       <c r="D14">
-        <v>0.857445490988495</v>
+        <v>0.806278469260452</v>
       </c>
       <c r="E14">
-        <v>0.833105542900532</v>
+        <v>0.862255928073848</v>
       </c>
       <c r="F14">
-        <v>0.827222990818765</v>
+        <v>0.873789460445227</v>
       </c>
       <c r="G14">
-        <v>0.857445490988495</v>
+        <v>0.806278469260452</v>
       </c>
       <c r="H14">
-        <v>0.84206314913502</v>
+        <v>0.838677551266768</v>
       </c>
       <c r="I14">
-        <v>0.908541319124791</v>
+        <v>0.903678794999893</v>
       </c>
       <c r="J14">
-        <v>0.917109732344243</v>
+        <v>0.908921835679264</v>
       </c>
       <c r="K14">
-        <v>0.8512256043899153</v>
+        <v>0.8189330001414494</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1000,31 +1000,31 @@
         </is>
       </c>
       <c r="C15">
-        <v>0.911772104137844</v>
+        <v>0.9187209156081</v>
       </c>
       <c r="D15">
-        <v>0.925830786239188</v>
+        <v>0.934486133768352</v>
       </c>
       <c r="E15">
-        <v>0.898612041151762</v>
+        <v>0.904059712361187</v>
       </c>
       <c r="F15">
-        <v>0.895264746572758</v>
+        <v>0.900578543579424</v>
       </c>
       <c r="G15">
-        <v>0.925830786239188</v>
+        <v>0.934486133768352</v>
       </c>
       <c r="H15">
-        <v>0.91029124972026</v>
+        <v>0.917219073237903</v>
       </c>
       <c r="I15">
-        <v>0.969513988399517</v>
+        <v>0.968160605248462</v>
       </c>
       <c r="J15">
-        <v>0.972086764935543</v>
+        <v>0.971696375712079</v>
       </c>
       <c r="K15">
-        <v>0.9195517375016145</v>
+        <v>0.9275018781896841</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1044,31 +1044,31 @@
         </is>
       </c>
       <c r="C16">
-        <v>0.679883033580682</v>
+        <v>0.687979499434033</v>
       </c>
       <c r="D16">
-        <v>0.6970177009435909</v>
+        <v>0.71608775797882</v>
       </c>
       <c r="E16">
-        <v>0.665490309516922</v>
+        <v>0.666342060599316</v>
       </c>
       <c r="F16">
-        <v>0.636397937366369</v>
+        <v>0.622940510627594</v>
       </c>
       <c r="G16">
-        <v>0.6970177009435909</v>
+        <v>0.71608775797882</v>
       </c>
       <c r="H16">
-        <v>0.6653298708129251</v>
+        <v>0.6662743185754399</v>
       </c>
       <c r="I16">
-        <v>0.7365554828727791</v>
+        <v>0.744059219798995</v>
       </c>
       <c r="J16">
-        <v>0.736419243605223</v>
+        <v>0.734255444536922</v>
       </c>
       <c r="K16">
-        <v>0.6839871313093081</v>
+        <v>0.6952945140097707</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1091,28 +1091,28 @@
         <v>0.83942271412401</v>
       </c>
       <c r="D17">
-        <v>0.870452985586822</v>
+        <v>0.880239520958084</v>
       </c>
       <c r="E17">
-        <v>0.813189044911222</v>
+        <v>0.806519393491964</v>
       </c>
       <c r="F17">
-        <v>0.797541189787448</v>
+        <v>0.785750220098101</v>
       </c>
       <c r="G17">
-        <v>0.870452985586822</v>
+        <v>0.880239520958084</v>
       </c>
       <c r="H17">
-        <v>0.832403517983723</v>
+        <v>0.830315313818653</v>
       </c>
       <c r="I17">
-        <v>0.90876721458836</v>
+        <v>0.90837170573169</v>
       </c>
       <c r="J17">
-        <v>0.91794749316845</v>
+        <v>0.918008926585313</v>
       </c>
       <c r="K17">
-        <v>0.854823272491979</v>
+        <v>0.8595663300404502</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1132,31 +1132,31 @@
         </is>
       </c>
       <c r="C18">
-        <v>0.808552114447414</v>
+        <v>0.788485725066029</v>
       </c>
       <c r="D18">
-        <v>0.8438441594842691</v>
+        <v>0.814040251916758</v>
       </c>
       <c r="E18">
-        <v>0.77982776320292</v>
+        <v>0.766777157478483</v>
       </c>
       <c r="F18">
-        <v>0.757247060303087</v>
+        <v>0.747799018991322</v>
       </c>
       <c r="G18">
-        <v>0.8438441594842691</v>
+        <v>0.814040251916758</v>
       </c>
       <c r="H18">
-        <v>0.798203751574203</v>
+        <v>0.779514913143232</v>
       </c>
       <c r="I18">
-        <v>0.832626044198133</v>
+        <v>0.836923133839624</v>
       </c>
       <c r="J18">
-        <v>0.660876150703164</v>
+        <v>0.666955776354443</v>
       </c>
       <c r="K18">
-        <v>0.824975680600655</v>
+        <v>0.7998695078967902</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1176,31 +1176,31 @@
         </is>
       </c>
       <c r="C19">
-        <v>0.911832654921498</v>
+        <v>0.902669475537668</v>
       </c>
       <c r="D19">
-        <v>0.935219311352392</v>
+        <v>0.906981917564433</v>
       </c>
       <c r="E19">
-        <v>0.890815230365242</v>
+        <v>0.898447465853583</v>
       </c>
       <c r="F19">
-        <v>0.885027494108405</v>
+        <v>0.897371399823922</v>
       </c>
       <c r="G19">
-        <v>0.935219311352392</v>
+        <v>0.906981917564433</v>
       </c>
       <c r="H19">
-        <v>0.909431403571083</v>
+        <v>0.902151064468714</v>
       </c>
       <c r="I19">
-        <v>0.960413866432291</v>
+        <v>0.95620650613656</v>
       </c>
       <c r="J19">
-        <v>0.592548014160434</v>
+        <v>0.5901779015815209</v>
       </c>
       <c r="K19">
-        <v>0.9247306179535497</v>
+        <v>0.9050433811964081</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1220,31 +1220,31 @@
         </is>
       </c>
       <c r="C20">
-        <v>0.838594031644302</v>
+        <v>0.856919687562588</v>
       </c>
       <c r="D20">
-        <v>0.784041532644885</v>
+        <v>0.852077455757887</v>
       </c>
       <c r="E20">
-        <v>0.868608153000714</v>
+        <v>0.8591192404030989</v>
       </c>
       <c r="F20">
-        <v>0.766523226304756</v>
+        <v>0.73314575747545</v>
       </c>
       <c r="G20">
-        <v>0.784041532644885</v>
+        <v>0.852077455757887</v>
       </c>
       <c r="H20">
-        <v>0.775183418417162</v>
+        <v>0.7881501690291201</v>
       </c>
       <c r="I20">
-        <v>0.8990840770929051</v>
+        <v>0.905879582105518</v>
       </c>
       <c r="J20">
-        <v>0.592607052373356</v>
+        <v>0.594953549722806</v>
       </c>
       <c r="K20">
-        <v>0.7804741040332551</v>
+        <v>0.8253012048192775</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1264,31 +1264,31 @@
         </is>
       </c>
       <c r="C21">
-        <v>0.927658722211096</v>
+        <v>0.918525936310835</v>
       </c>
       <c r="D21">
-        <v>0.901560424966799</v>
+        <v>0.882801437751879</v>
       </c>
       <c r="E21">
-        <v>0.94246343147718</v>
+        <v>0.939305625950329</v>
       </c>
       <c r="F21">
-        <v>0.898874544852698</v>
+        <v>0.894295487145537</v>
       </c>
       <c r="G21">
-        <v>0.901560424966799</v>
+        <v>0.882801437751879</v>
       </c>
       <c r="H21">
-        <v>0.900215481518316</v>
+        <v>0.888511291383469</v>
       </c>
       <c r="I21">
-        <v>0.968450550828447</v>
+        <v>0.961612670487127</v>
       </c>
       <c r="J21">
-        <v>0.515518545121373</v>
+        <v>0.547195637495539</v>
       </c>
       <c r="K21">
-        <v>0.9010219656247924</v>
+        <v>0.8850765501124774</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1308,31 +1308,31 @@
         </is>
       </c>
       <c r="C22">
-        <v>0.885674757892089</v>
+        <v>0.846324361715508</v>
       </c>
       <c r="D22">
-        <v>0.88195179672417</v>
+        <v>0.853017531489375</v>
       </c>
       <c r="E22">
-        <v>0.889471010351178</v>
+        <v>0.839880272780572</v>
       </c>
       <c r="F22">
-        <v>0.890548358697019</v>
+        <v>0.836844422085272</v>
       </c>
       <c r="G22">
-        <v>0.88195179672417</v>
+        <v>0.853017531489375</v>
       </c>
       <c r="H22">
-        <v>0.886229231202478</v>
+        <v>0.844853583048964</v>
       </c>
       <c r="I22">
-        <v>0.943052886314698</v>
+        <v>0.910943958191856</v>
       </c>
       <c r="J22">
-        <v>0.630793065538197</v>
+        <v>0.601180202906297</v>
       </c>
       <c r="K22">
-        <v>0.8836578060651441</v>
+        <v>0.8497330915406617</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1352,31 +1352,31 @@
         </is>
       </c>
       <c r="C23">
-        <v>0.92142497799019</v>
+        <v>0.9071814866054581</v>
       </c>
       <c r="D23">
-        <v>0.929363147104049</v>
+        <v>0.936232567540255</v>
       </c>
       <c r="E23">
-        <v>0.913775006174364</v>
+        <v>0.881758151052414</v>
       </c>
       <c r="F23">
-        <v>0.912180857753742</v>
+        <v>0.873883788202742</v>
       </c>
       <c r="G23">
-        <v>0.929363147104049</v>
+        <v>0.936232567540255</v>
       </c>
       <c r="H23">
-        <v>0.920691843859092</v>
+        <v>0.903984387705318</v>
       </c>
       <c r="I23">
-        <v>0.962655203130652</v>
+        <v>0.956357819873521</v>
       </c>
       <c r="J23">
-        <v>0.585344407388666</v>
+        <v>0.578929268146042</v>
       </c>
       <c r="K23">
-        <v>0.925875098935328</v>
+        <v>0.9230610835082502</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1396,31 +1396,31 @@
         </is>
       </c>
       <c r="C24">
-        <v>0.6649792478933469</v>
+        <v>0.67214815746447</v>
       </c>
       <c r="D24">
-        <v>0.716406829992576</v>
+        <v>0.716027462121212</v>
       </c>
       <c r="E24">
-        <v>0.633301153396677</v>
+        <v>0.643084883964039</v>
       </c>
       <c r="F24">
-        <v>0.546157716010565</v>
+        <v>0.570588605206892</v>
       </c>
       <c r="G24">
-        <v>0.716406829992576</v>
+        <v>0.716027462121212</v>
       </c>
       <c r="H24">
-        <v>0.619803746654773</v>
+        <v>0.635087842094212</v>
       </c>
       <c r="I24">
-        <v>0.740819620105545</v>
+        <v>0.74101841111894</v>
       </c>
       <c r="J24">
-        <v>0.708685169616008</v>
+        <v>0.709162220117423</v>
       </c>
       <c r="K24">
-        <v>0.6743640711867565</v>
+        <v>0.6812959903889473</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1440,31 +1440,31 @@
         </is>
       </c>
       <c r="C25">
-        <v>0.826342598415294</v>
+        <v>0.827584580555905</v>
       </c>
       <c r="D25">
-        <v>0.909492622109998</v>
+        <v>0.909612738352664</v>
       </c>
       <c r="E25">
-        <v>0.771261303643301</v>
+        <v>0.772928509679616</v>
       </c>
       <c r="F25">
-        <v>0.724814488743554</v>
+        <v>0.727455665953968</v>
       </c>
       <c r="G25">
-        <v>0.909492622109998</v>
+        <v>0.909612738352664</v>
       </c>
       <c r="H25">
-        <v>0.806719160104987</v>
+        <v>0.808399867223397</v>
       </c>
       <c r="I25">
-        <v>0.89737090797741</v>
+        <v>0.898746828079375</v>
       </c>
       <c r="J25">
-        <v>0.678384506532193</v>
+        <v>0.6818353303525549</v>
       </c>
       <c r="K25">
-        <v>0.8653932786737546</v>
+        <v>0.8662313544599535</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1484,31 +1484,31 @@
         </is>
       </c>
       <c r="C26">
-        <v>0.732023266781953</v>
+        <v>0.6910765941391021</v>
       </c>
       <c r="D26">
-        <v>0.717583583937732</v>
+        <v>0.674556213017751</v>
       </c>
       <c r="E26">
-        <v>0.74851811935875</v>
+        <v>0.711050913384733</v>
       </c>
       <c r="F26">
-        <v>0.765232974910394</v>
+        <v>0.738397685825682</v>
       </c>
       <c r="G26">
-        <v>0.717583583937732</v>
+        <v>0.674556213017751</v>
       </c>
       <c r="H26">
-        <v>0.740642687602702</v>
+        <v>0.705034675312978</v>
       </c>
       <c r="I26">
-        <v>0.7718260252760351</v>
+        <v>0.73148824135476</v>
       </c>
       <c r="J26">
         <v>1</v>
       </c>
       <c r="K26">
-        <v>0.7266327517644108</v>
+        <v>0.6864258155033318</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1528,31 +1528,31 @@
         </is>
       </c>
       <c r="C27">
-        <v>0.710305049584309</v>
+        <v>0.703244874858508</v>
       </c>
       <c r="D27">
-        <v>0.707126948775056</v>
+        <v>0.703015075376884</v>
       </c>
       <c r="E27">
-        <v>0.713587425321875</v>
+        <v>0.7034751951649461</v>
       </c>
       <c r="F27">
-        <v>0.718303220738413</v>
+        <v>0.703810841403597</v>
       </c>
       <c r="G27">
-        <v>0.707126948775056</v>
+        <v>0.703015075376884</v>
       </c>
       <c r="H27">
-        <v>0.712671270244571</v>
+        <v>0.703412733329143</v>
       </c>
       <c r="I27">
-        <v>0.782981531716801</v>
+        <v>0.782782402429002</v>
       </c>
       <c r="J27">
         <v>1</v>
       </c>
       <c r="K27">
-        <v>0.7093342931790962</v>
+        <v>0.7031740845919928</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1572,31 +1572,31 @@
         </is>
       </c>
       <c r="C28">
-        <v>0.668215501702383</v>
+        <v>0.6625275385539759</v>
       </c>
       <c r="D28">
-        <v>0.537392138063279</v>
+        <v>0.527681360638667</v>
       </c>
       <c r="E28">
-        <v>0.762091503267974</v>
+        <v>0.778141507328324</v>
       </c>
       <c r="F28">
-        <v>0.618448637316562</v>
+        <v>0.6709698775239989</v>
       </c>
       <c r="G28">
-        <v>0.537392138063279</v>
+        <v>0.527681360638667</v>
       </c>
       <c r="H28">
-        <v>0.575078233211922</v>
+        <v>0.590761159955312</v>
       </c>
       <c r="I28">
-        <v>0.732985899178091</v>
+        <v>0.73916932844479</v>
       </c>
       <c r="J28">
         <v>1</v>
       </c>
       <c r="K28">
-        <v>0.5518579052044976</v>
+        <v>0.5512246414909624</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1616,31 +1616,31 @@
         </is>
       </c>
       <c r="C29">
-        <v>0.8389745643901459</v>
+        <v>0.837832966152614</v>
       </c>
       <c r="D29">
-        <v>0.830039267015707</v>
+        <v>0.813269194727307</v>
       </c>
       <c r="E29">
-        <v>0.842914862914863</v>
+        <v>0.84942369483831</v>
       </c>
       <c r="F29">
-        <v>0.699713119276178</v>
+        <v>0.718194858214719</v>
       </c>
       <c r="G29">
-        <v>0.830039267015707</v>
+        <v>0.813269194727307</v>
       </c>
       <c r="H29">
-        <v>0.759324672214572</v>
+        <v>0.762780886532095</v>
       </c>
       <c r="I29">
-        <v>0.8716294574904631</v>
+        <v>0.873765299994187</v>
       </c>
       <c r="J29">
         <v>1</v>
       </c>
       <c r="K29">
-        <v>0.8002296645887491</v>
+        <v>0.7922925237967721</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1660,31 +1660,31 @@
         </is>
       </c>
       <c r="C30">
-        <v>0.669208275688593</v>
+        <v>0.68785372909068</v>
       </c>
       <c r="D30">
-        <v>0.615629230141166</v>
+        <v>0.684506346314197</v>
       </c>
       <c r="E30">
-        <v>0.815316107107283</v>
+        <v>0.691324815063887</v>
       </c>
       <c r="F30">
-        <v>0.9008929694378069</v>
+        <v>0.696924915105018</v>
       </c>
       <c r="G30">
-        <v>0.615629230141166</v>
+        <v>0.684506346314197</v>
       </c>
       <c r="H30">
-        <v>0.731431488927181</v>
+        <v>0.6906598114824331</v>
       </c>
       <c r="I30">
-        <v>0.741204750259343</v>
+        <v>0.7610761110716801</v>
       </c>
       <c r="J30">
         <v>1</v>
       </c>
       <c r="K30">
-        <v>0.6572524407252442</v>
+        <v>0.6869545274223945</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -1704,31 +1704,31 @@
         </is>
       </c>
       <c r="C31">
-        <v>0.834879260470381</v>
+        <v>0.839894352911583</v>
       </c>
       <c r="D31">
-        <v>0.836391775370329</v>
+        <v>0.824858757062147</v>
       </c>
       <c r="E31">
-        <v>0.833380286098851</v>
+        <v>0.856389291837004</v>
       </c>
       <c r="F31">
-        <v>0.832631115582946</v>
+        <v>0.863036096088542</v>
       </c>
       <c r="G31">
-        <v>0.836391775370329</v>
+        <v>0.824858757062147</v>
       </c>
       <c r="H31">
-        <v>0.834507208697707</v>
+        <v>0.843515673017824</v>
       </c>
       <c r="I31">
-        <v>0.899203616562526</v>
+        <v>0.901708094550667</v>
       </c>
       <c r="J31">
         <v>1</v>
       </c>
       <c r="K31">
-        <v>0.8356369282035745</v>
+        <v>0.8322216023479759</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -1748,31 +1748,31 @@
         </is>
       </c>
       <c r="C32">
-        <v>0.653990064142875</v>
+        <v>0.6604200729467991</v>
       </c>
       <c r="D32">
-        <v>0.696505236127272</v>
+        <v>0.651116640009478</v>
       </c>
       <c r="E32">
-        <v>0.6265994571539359</v>
+        <v>0.67094418012464</v>
       </c>
       <c r="F32">
-        <v>0.545811847566344</v>
+        <v>0.691202364482455</v>
       </c>
       <c r="G32">
-        <v>0.696505236127272</v>
+        <v>0.651116640009478</v>
       </c>
       <c r="H32">
-        <v>0.61201896803991</v>
+        <v>0.670560961473935</v>
       </c>
       <c r="I32">
-        <v>0.7237429282061409</v>
+        <v>0.729044718720424</v>
       </c>
       <c r="J32">
         <v>1</v>
       </c>
       <c r="K32">
-        <v>0.6600581006266351</v>
+        <v>0.6587574617025866</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -1792,31 +1792,31 @@
         </is>
       </c>
       <c r="C33">
-        <v>0.806046409256697</v>
+        <v>0.806832473902654</v>
       </c>
       <c r="D33">
-        <v>0.874437391806117</v>
+        <v>0.873702753417838</v>
       </c>
       <c r="E33">
-        <v>0.758780208970303</v>
+        <v>0.760261368182424</v>
       </c>
       <c r="F33">
-        <v>0.714721418689473</v>
+        <v>0.717362595899887</v>
       </c>
       <c r="G33">
-        <v>0.874437391806117</v>
+        <v>0.873702753417838</v>
       </c>
       <c r="H33">
-        <v>0.786553400577865</v>
+        <v>0.787851580710327</v>
       </c>
       <c r="I33">
-        <v>0.862994249589609</v>
+        <v>0.862675362016037</v>
       </c>
       <c r="J33">
         <v>1</v>
       </c>
       <c r="K33">
-        <v>0.8370279267071236</v>
+        <v>0.8372108384217944</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -1836,31 +1836,31 @@
         </is>
       </c>
       <c r="C34">
-        <v>0.712309385316774</v>
+        <v>0.694440950823796</v>
       </c>
       <c r="D34">
-        <v>0.690762711864407</v>
+        <v>0.664441844386534</v>
       </c>
       <c r="E34">
-        <v>0.739347749025168</v>
+        <v>0.7378278593954311</v>
       </c>
       <c r="F34">
-        <v>0.768817204301075</v>
+        <v>0.785655892340586</v>
       </c>
       <c r="G34">
-        <v>0.690762711864407</v>
+        <v>0.664441844386534</v>
       </c>
       <c r="H34">
-        <v>0.727702883671101</v>
+        <v>0.719982711424867</v>
       </c>
       <c r="I34">
-        <v>0.706528405235605</v>
+        <v>0.684420087297842</v>
       </c>
       <c r="J34">
-        <v>0.993457729663883</v>
+        <v>0.998845438217405</v>
       </c>
       <c r="K34">
-        <v>0.7050794090169892</v>
+        <v>0.6855971639923611</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -1880,31 +1880,31 @@
         </is>
       </c>
       <c r="C35">
-        <v>0.6993666409970301</v>
+        <v>0.690164759149792</v>
       </c>
       <c r="D35">
-        <v>0.713392496974587</v>
+        <v>0.690848848217103</v>
       </c>
       <c r="E35">
-        <v>0.687051739913226</v>
+        <v>0.689485556739144</v>
       </c>
       <c r="F35">
-        <v>0.6668342498036131</v>
+        <v>0.688372531757012</v>
       </c>
       <c r="G35">
-        <v>0.713392496974587</v>
+        <v>0.690848848217103</v>
       </c>
       <c r="H35">
-        <v>0.689328114595683</v>
+        <v>0.689608466941758</v>
       </c>
       <c r="I35">
-        <v>0.759948905427519</v>
+        <v>0.7536074949522999</v>
       </c>
       <c r="J35">
-        <v>0.991380711872582</v>
+        <v>0.991120094300009</v>
       </c>
       <c r="K35">
-        <v>0.7035679001704054</v>
+        <v>0.6903521606417597</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -1924,31 +1924,31 @@
         </is>
       </c>
       <c r="C36">
-        <v>0.6881434007610659</v>
+        <v>0.6871419987983181</v>
       </c>
       <c r="D36">
-        <v>0.61608359836438</v>
+        <v>0.613811903680145</v>
       </c>
       <c r="E36">
-        <v>0.708516377649326</v>
+        <v>0.707874116891458</v>
       </c>
       <c r="F36">
-        <v>0.37404832836809</v>
+        <v>0.372669094118945</v>
       </c>
       <c r="G36">
-        <v>0.61608359836438</v>
+        <v>0.613811903680145</v>
       </c>
       <c r="H36">
-        <v>0.465483505543922</v>
+        <v>0.463767120936459</v>
       </c>
       <c r="I36">
-        <v>0.676587752229176</v>
+        <v>0.6763707097453751</v>
       </c>
       <c r="J36">
-        <v>0.99324713615384</v>
+        <v>0.990978466347301</v>
       </c>
       <c r="K36">
-        <v>0.5454896533968397</v>
+        <v>0.543478260869565</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -1968,31 +1968,31 @@
         </is>
       </c>
       <c r="C37">
-        <v>0.785439615461646</v>
+        <v>0.784818746244743</v>
       </c>
       <c r="D37">
-        <v>0.689271306745647</v>
+        <v>0.686697015680324</v>
       </c>
       <c r="E37">
-        <v>0.847497281444624</v>
+        <v>0.849137931034483</v>
       </c>
       <c r="F37">
-        <v>0.744676155798301</v>
+        <v>0.748979366655633</v>
       </c>
       <c r="G37">
-        <v>0.689271306745647</v>
+        <v>0.686697015680324</v>
       </c>
       <c r="H37">
-        <v>0.715903365244371</v>
+        <v>0.716487228203504</v>
       </c>
       <c r="I37">
-        <v>0.7967913293900309</v>
+        <v>0.797581192958143</v>
       </c>
       <c r="J37">
-        <v>0.9809291308608989</v>
+        <v>0.979788445168103</v>
       </c>
       <c r="K37">
-        <v>0.6996827634825522</v>
+        <v>0.6983108038598443</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2012,31 +2012,31 @@
         </is>
       </c>
       <c r="C38">
-        <v>0.6351873978115961</v>
+        <v>0.634464218337316</v>
       </c>
       <c r="D38">
-        <v>0.73062275384863</v>
+        <v>0.6026450327628829</v>
       </c>
       <c r="E38">
-        <v>0.595618814633604</v>
+        <v>0.694873547505126</v>
       </c>
       <c r="F38">
-        <v>0.42827946170293</v>
+        <v>0.789460445227015</v>
       </c>
       <c r="G38">
-        <v>0.73062275384863</v>
+        <v>0.6026450327628829</v>
       </c>
       <c r="H38">
-        <v>0.5400122901262711</v>
+        <v>0.683517769883077</v>
       </c>
       <c r="I38">
-        <v>0.687787141476419</v>
+        <v>0.699292649382258</v>
       </c>
       <c r="J38">
-        <v>0.98430594625767</v>
+        <v>0.988804869046999</v>
       </c>
       <c r="K38">
-        <v>0.640228999022336</v>
+        <v>0.6325835449671462</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2056,31 +2056,31 @@
         </is>
       </c>
       <c r="C39">
-        <v>0.797997107282103</v>
+        <v>0.801911709218966</v>
       </c>
       <c r="D39">
-        <v>0.787379847781922</v>
+        <v>0.791146149181322</v>
       </c>
       <c r="E39">
-        <v>0.809428972542362</v>
+        <v>0.81350398328327</v>
       </c>
       <c r="F39">
-        <v>0.81646962646208</v>
+        <v>0.820399949691863</v>
       </c>
       <c r="G39">
-        <v>0.787379847781922</v>
+        <v>0.791146149181322</v>
       </c>
       <c r="H39">
-        <v>0.801660929564855</v>
+        <v>0.805507532724129</v>
       </c>
       <c r="I39">
-        <v>0.813660926824138</v>
+        <v>0.813118803712704</v>
       </c>
       <c r="J39">
-        <v>0.985726981818895</v>
+        <v>0.987384762123839</v>
       </c>
       <c r="K39">
-        <v>0.7930307842658197</v>
+        <v>0.7968288094598227</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2100,31 +2100,31 @@
         </is>
       </c>
       <c r="C40">
-        <v>0.630549616400453</v>
+        <v>0.6311941894101371</v>
       </c>
       <c r="D40">
-        <v>0.737773450922002</v>
+        <v>0.741534008683068</v>
       </c>
       <c r="E40">
-        <v>0.589975295800286</v>
+        <v>0.590054604709386</v>
       </c>
       <c r="F40">
-        <v>0.405074833354295</v>
+        <v>0.402779524588102</v>
       </c>
       <c r="G40">
-        <v>0.737773450922002</v>
+        <v>0.741534008683068</v>
       </c>
       <c r="H40">
-        <v>0.522997604839037</v>
+        <v>0.522015525988712</v>
       </c>
       <c r="I40">
-        <v>0.689928509699257</v>
+        <v>0.691915028822067</v>
       </c>
       <c r="J40">
-        <v>0.998879021806576</v>
+        <v>0.998874223816725</v>
       </c>
       <c r="K40">
-        <v>0.6336815802935505</v>
+        <v>0.6347617537461347</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2144,31 +2144,31 @@
         </is>
       </c>
       <c r="C41">
-        <v>0.782322978241731</v>
+        <v>0.783046157716011</v>
       </c>
       <c r="D41">
-        <v>0.807985182136242</v>
+        <v>0.809262058540607</v>
       </c>
       <c r="E41">
-        <v>0.7606083473617</v>
+        <v>0.760927536231884</v>
       </c>
       <c r="F41">
         <v>0.740661552006037</v>
       </c>
       <c r="G41">
-        <v>0.807985182136242</v>
+        <v>0.809262058540607</v>
       </c>
       <c r="H41">
-        <v>0.772860001968569</v>
+        <v>0.77344365642238</v>
       </c>
       <c r="I41">
-        <v>0.8004955728791689</v>
+        <v>0.801774445979739</v>
       </c>
       <c r="J41">
-        <v>0.987022231644782</v>
+        <v>0.987375690935425</v>
       </c>
       <c r="K41">
-        <v>0.7935588195660962</v>
+        <v>0.7945438355055449</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2188,31 +2188,31 @@
         </is>
       </c>
       <c r="C42">
-        <v>0.782974375098255</v>
+        <v>0.7322034964155451</v>
       </c>
       <c r="D42">
-        <v>0.800487430307482</v>
+        <v>0.760328539199098</v>
       </c>
       <c r="E42">
-        <v>0.767388656148795</v>
+        <v>0.7095629965947789</v>
       </c>
       <c r="F42">
-        <v>0.753851474564548</v>
+        <v>0.678185133945416</v>
       </c>
       <c r="G42">
-        <v>0.800487430307482</v>
+        <v>0.760328539199098</v>
       </c>
       <c r="H42">
-        <v>0.7764698262601401</v>
+        <v>0.716911520308449</v>
       </c>
       <c r="I42">
-        <v>0.793038666064696</v>
+        <v>0.762224571687601</v>
       </c>
       <c r="J42">
-        <v>0.71232840802571</v>
+        <v>0.712317927548219</v>
       </c>
       <c r="K42">
-        <v>0.7907042699415641</v>
+        <v>0.7423456042291918</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2232,31 +2232,31 @@
         </is>
       </c>
       <c r="C43">
-        <v>0.770969212151692</v>
+        <v>0.771365237077097</v>
       </c>
       <c r="D43">
-        <v>0.794724613912806</v>
+        <v>0.781004786246866</v>
       </c>
       <c r="E43">
-        <v>0.750734844736766</v>
+        <v>0.762365101079191</v>
       </c>
       <c r="F43">
-        <v>0.730871956009427</v>
+        <v>0.754213306502327</v>
       </c>
       <c r="G43">
-        <v>0.794724613912806</v>
+        <v>0.781004786246866</v>
       </c>
       <c r="H43">
-        <v>0.761462033293503</v>
+        <v>0.767375273925492</v>
       </c>
       <c r="I43">
-        <v>0.843754714041414</v>
+        <v>0.849201642552617</v>
       </c>
       <c r="J43">
-        <v>0.712427934227307</v>
+        <v>0.712317927548219</v>
       </c>
       <c r="K43">
-        <v>0.7810768517834479</v>
+        <v>0.7754952927788122</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2276,31 +2276,31 @@
         </is>
       </c>
       <c r="C44">
-        <v>0.702323252553575</v>
+        <v>0.7086721409973959</v>
       </c>
       <c r="D44">
-        <v>0.608643537324366</v>
+        <v>0.624322822614252</v>
       </c>
       <c r="E44">
-        <v>0.742617363159854</v>
+        <v>0.74285151412811</v>
       </c>
       <c r="F44">
-        <v>0.504248041487366</v>
+        <v>0.495917466622531</v>
       </c>
       <c r="G44">
-        <v>0.608643537324366</v>
+        <v>0.624322822614252</v>
       </c>
       <c r="H44">
-        <v>0.551549346770057</v>
+        <v>0.552761038002706</v>
       </c>
       <c r="I44">
-        <v>0.726446857838976</v>
+        <v>0.733385640328209</v>
       </c>
       <c r="J44">
         <v>0.61656169060112</v>
       </c>
       <c r="K44">
-        <v>0.584443819218866</v>
+        <v>0.5935840883277425</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2320,31 +2320,31 @@
         </is>
       </c>
       <c r="C45">
-        <v>0.838854396154616</v>
+        <v>0.840476667334268</v>
       </c>
       <c r="D45">
-        <v>0.7845528455284549</v>
+        <v>0.785181027224249</v>
       </c>
       <c r="E45">
-        <v>0.868706934012043</v>
+        <v>0.87115055270123</v>
       </c>
       <c r="F45">
-        <v>0.766633565044687</v>
+        <v>0.77170914708154</v>
       </c>
       <c r="G45">
-        <v>0.7845528455284549</v>
+        <v>0.785181027224249</v>
       </c>
       <c r="H45">
-        <v>0.7754897036664991</v>
+        <v>0.778386800589856</v>
       </c>
       <c r="I45">
-        <v>0.891360887432656</v>
+        <v>0.893733642170786</v>
       </c>
       <c r="J45">
         <v>0.61656169060112</v>
       </c>
       <c r="K45">
-        <v>0.7809022860610962</v>
+        <v>0.7824491531112252</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2364,31 +2364,31 @@
         </is>
       </c>
       <c r="C46">
-        <v>0.7168752358193941</v>
+        <v>0.7081027543705189</v>
       </c>
       <c r="D46">
-        <v>0.792428032390724</v>
+        <v>0.742533621605775</v>
       </c>
       <c r="E46">
-        <v>0.672347017815647</v>
+        <v>0.682232440320493</v>
       </c>
       <c r="F46">
-        <v>0.587693371902905</v>
+        <v>0.637121116840649</v>
       </c>
       <c r="G46">
-        <v>0.792428032390724</v>
+        <v>0.742533621605775</v>
       </c>
       <c r="H46">
-        <v>0.674874979689841</v>
+        <v>0.6858003486030499</v>
       </c>
       <c r="I46">
-        <v>0.773382988206234</v>
+        <v>0.752443621003638</v>
       </c>
       <c r="J46">
         <v>0.712317927548219</v>
       </c>
       <c r="K46">
-        <v>0.7408126704293235</v>
+        <v>0.7187499999999998</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2408,31 +2408,31 @@
         </is>
       </c>
       <c r="C47">
-        <v>0.8588227895862161</v>
+        <v>0.865645830713118</v>
       </c>
       <c r="D47">
-        <v>0.870832520959251</v>
+        <v>0.885832780358328</v>
       </c>
       <c r="E47">
-        <v>0.8475665468721451</v>
+        <v>0.847466236404924</v>
       </c>
       <c r="F47">
-        <v>0.8426298578795119</v>
+        <v>0.839485599295686</v>
       </c>
       <c r="G47">
-        <v>0.870832520959251</v>
+        <v>0.885832780358328</v>
       </c>
       <c r="H47">
-        <v>0.856499089136757</v>
+        <v>0.862036678290068</v>
       </c>
       <c r="I47">
-        <v>0.911142361165541</v>
+        <v>0.9149551133063299</v>
       </c>
       <c r="J47">
         <v>0.712317927548219</v>
       </c>
       <c r="K47">
-        <v>0.8650419625564878</v>
+        <v>0.8761584101231263</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -2452,31 +2452,31 @@
         </is>
       </c>
       <c r="C48">
-        <v>0.653109671739404</v>
+        <v>0.652983901396051</v>
       </c>
       <c r="D48">
-        <v>0.695522987351937</v>
+        <v>0.704802794965694</v>
       </c>
       <c r="E48">
-        <v>0.625817120119887</v>
+        <v>0.622092293794384</v>
       </c>
       <c r="F48">
-        <v>0.5446484718903279</v>
+        <v>0.526474657275814</v>
       </c>
       <c r="G48">
-        <v>0.695522987351937</v>
+        <v>0.704802794965694</v>
       </c>
       <c r="H48">
-        <v>0.610908321430461</v>
+        <v>0.60272493295657</v>
       </c>
       <c r="I48">
-        <v>0.714529373635217</v>
+        <v>0.712405743028837</v>
       </c>
       <c r="J48">
         <v>0.712317927548219</v>
       </c>
       <c r="K48">
-        <v>0.6590120525931333</v>
+        <v>0.6600857827677554</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2496,31 +2496,31 @@
         </is>
       </c>
       <c r="C49">
-        <v>0.807021129417683</v>
+        <v>0.807854357942397</v>
       </c>
       <c r="D49">
-        <v>0.86436061047054</v>
+        <v>0.8559328195434061</v>
       </c>
       <c r="E49">
-        <v>0.765274796924665</v>
+        <v>0.771218836565097</v>
       </c>
       <c r="F49">
-        <v>0.728336058357439</v>
+        <v>0.740315683561816</v>
       </c>
       <c r="G49">
-        <v>0.86436061047054</v>
+        <v>0.8559328195434061</v>
       </c>
       <c r="H49">
-        <v>0.790539733460744</v>
+        <v>0.793937145940113</v>
       </c>
       <c r="I49">
-        <v>0.861478169544339</v>
+        <v>0.860876842942453</v>
       </c>
       <c r="J49">
         <v>0.712317927548219</v>
       </c>
       <c r="K49">
-        <v>0.8332374100719424</v>
+        <v>0.8300078964437804</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>

</xml_diff>